<commit_message>
Updated BMS performance data and dashboard inputs
</commit_message>
<xml_diff>
--- a/data/JFMP_RR.xlsx
+++ b/data/JFMP_RR.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pb0e\Downloads\Phils Scripts\jfmp_dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pb0e\Downloads\git_dashboard\streamlit-test\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94092296-685D-4833-9F46-EDD9801B8A03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D17A3FB-F61D-4E86-A2D0-3AEA72C1E94F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{67390A52-5801-4610-A7E5-7A5F58273BD5}"/>
+    <workbookView xWindow="3216" yWindow="2556" windowWidth="17280" windowHeight="8976" activeTab="1" xr2:uid="{67390A52-5801-4610-A7E5-7A5F58273BD5}"/>
   </bookViews>
   <sheets>
     <sheet name="Murray Goldfields" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="7">
   <si>
     <t>Season</t>
   </si>
@@ -6076,15 +6076,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA9F743B-C2DA-4E63-8B3A-4D852F0FC056}">
   <dimension ref="A1:G83"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="13.28515625" customWidth="1"/>
-    <col min="5" max="5" width="34.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.85546875" customWidth="1"/>
-    <col min="7" max="7" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" customWidth="1"/>
+    <col min="5" max="5" width="34.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.88671875" customWidth="1"/>
+    <col min="7" max="7" width="38.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6107,7 +6107,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1980</v>
       </c>
@@ -6122,7 +6122,7 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>1981</v>
       </c>
@@ -6137,7 +6137,7 @@
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>1982</v>
       </c>
@@ -6152,7 +6152,7 @@
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>1983</v>
       </c>
@@ -6167,7 +6167,7 @@
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>1984</v>
       </c>
@@ -6182,7 +6182,7 @@
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>1985</v>
       </c>
@@ -6197,7 +6197,7 @@
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>1986</v>
       </c>
@@ -6212,7 +6212,7 @@
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>1987</v>
       </c>
@@ -6227,7 +6227,7 @@
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>1988</v>
       </c>
@@ -6242,7 +6242,7 @@
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>1989</v>
       </c>
@@ -6257,7 +6257,7 @@
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>1990</v>
       </c>
@@ -6272,7 +6272,7 @@
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>1991</v>
       </c>
@@ -6287,7 +6287,7 @@
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>1992</v>
       </c>
@@ -6302,7 +6302,7 @@
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>1993</v>
       </c>
@@ -6317,7 +6317,7 @@
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>1994</v>
       </c>
@@ -6332,7 +6332,7 @@
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>1995</v>
       </c>
@@ -6347,7 +6347,7 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>1996</v>
       </c>
@@ -6362,7 +6362,7 @@
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>1997</v>
       </c>
@@ -6377,7 +6377,7 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>1998</v>
       </c>
@@ -6392,7 +6392,7 @@
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>1999</v>
       </c>
@@ -6407,7 +6407,7 @@
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>2000</v>
       </c>
@@ -6422,7 +6422,7 @@
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>2001</v>
       </c>
@@ -6437,7 +6437,7 @@
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>2002</v>
       </c>
@@ -6452,7 +6452,7 @@
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>2003</v>
       </c>
@@ -6467,7 +6467,7 @@
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>2004</v>
       </c>
@@ -6482,7 +6482,7 @@
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>2005</v>
       </c>
@@ -6497,7 +6497,7 @@
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>2006</v>
       </c>
@@ -6512,7 +6512,7 @@
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>2007</v>
       </c>
@@ -6527,7 +6527,7 @@
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>2008</v>
       </c>
@@ -6542,7 +6542,7 @@
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>2009</v>
       </c>
@@ -6557,7 +6557,7 @@
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>2010</v>
       </c>
@@ -6572,7 +6572,7 @@
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>2011</v>
       </c>
@@ -6587,7 +6587,7 @@
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>2012</v>
       </c>
@@ -6602,7 +6602,7 @@
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>2013</v>
       </c>
@@ -6617,7 +6617,7 @@
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>2014</v>
       </c>
@@ -6632,7 +6632,7 @@
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
         <v>2015</v>
       </c>
@@ -6647,7 +6647,7 @@
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>2016</v>
       </c>
@@ -6662,7 +6662,7 @@
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
         <v>2017</v>
       </c>
@@ -6677,7 +6677,7 @@
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>2018</v>
       </c>
@@ -6692,7 +6692,7 @@
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>2019</v>
       </c>
@@ -6707,7 +6707,7 @@
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>2020</v>
       </c>
@@ -6726,7 +6726,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <v>2021</v>
       </c>
@@ -6745,7 +6745,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
         <v>2022</v>
       </c>
@@ -6760,7 +6760,7 @@
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
         <v>2023</v>
       </c>
@@ -6775,7 +6775,7 @@
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
         <v>2024</v>
       </c>
@@ -6790,7 +6790,7 @@
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <v>2025</v>
       </c>
@@ -6809,7 +6809,7 @@
         <v>74.099999999999994</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>2026</v>
       </c>
@@ -6828,7 +6828,7 @@
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
         <v>2027</v>
       </c>
@@ -6845,7 +6845,7 @@
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
         <v>2028</v>
       </c>
@@ -6862,7 +6862,7 @@
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
         <v>2029</v>
       </c>
@@ -6879,7 +6879,7 @@
       <c r="F51" s="1"/>
       <c r="G51" s="1"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
         <v>2030</v>
       </c>
@@ -6896,7 +6896,7 @@
         <v>76.760000000000005</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
         <v>2031</v>
       </c>
@@ -6909,7 +6909,7 @@
       <c r="F53" s="1"/>
       <c r="G53" s="1"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
         <v>2032</v>
       </c>
@@ -6922,7 +6922,7 @@
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
         <v>2033</v>
       </c>
@@ -6935,7 +6935,7 @@
       <c r="F55" s="1"/>
       <c r="G55" s="1"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
         <v>2034</v>
       </c>
@@ -6948,7 +6948,7 @@
       <c r="F56" s="1"/>
       <c r="G56" s="1"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
         <v>2035</v>
       </c>
@@ -6965,7 +6965,7 @@
         <v>75.42</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
         <v>2036</v>
       </c>
@@ -6978,7 +6978,7 @@
       <c r="F58" s="1"/>
       <c r="G58" s="1"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
         <v>2037</v>
       </c>
@@ -6991,7 +6991,7 @@
       <c r="F59" s="1"/>
       <c r="G59" s="1"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
         <v>2038</v>
       </c>
@@ -7004,7 +7004,7 @@
       <c r="F60" s="1"/>
       <c r="G60" s="1"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
         <v>2039</v>
       </c>
@@ -7017,7 +7017,7 @@
       <c r="F61" s="1"/>
       <c r="G61" s="1"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="2">
         <v>2040</v>
       </c>
@@ -7034,7 +7034,7 @@
         <v>80.2</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
         <v>2041</v>
       </c>
@@ -7047,7 +7047,7 @@
       <c r="F63" s="1"/>
       <c r="G63" s="1"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
         <v>2042</v>
       </c>
@@ -7060,7 +7060,7 @@
       <c r="F64" s="1"/>
       <c r="G64" s="1"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
         <v>2043</v>
       </c>
@@ -7073,7 +7073,7 @@
       <c r="F65" s="1"/>
       <c r="G65" s="1"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
         <v>2044</v>
       </c>
@@ -7086,7 +7086,7 @@
       <c r="F66" s="1"/>
       <c r="G66" s="1"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
         <v>2045</v>
       </c>
@@ -7103,7 +7103,7 @@
         <v>78.5</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" s="2">
         <v>2046</v>
       </c>
@@ -7116,7 +7116,7 @@
       <c r="F68" s="1"/>
       <c r="G68" s="1"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
         <v>2047</v>
       </c>
@@ -7129,7 +7129,7 @@
       <c r="F69" s="1"/>
       <c r="G69" s="1"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="2">
         <v>2048</v>
       </c>
@@ -7142,7 +7142,7 @@
       <c r="F70" s="1"/>
       <c r="G70" s="1"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="2">
         <v>2049</v>
       </c>
@@ -7155,7 +7155,7 @@
       <c r="F71" s="1"/>
       <c r="G71" s="1"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="2">
         <v>2050</v>
       </c>
@@ -7172,7 +7172,7 @@
         <v>83.75</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="2">
         <v>2051</v>
       </c>
@@ -7185,7 +7185,7 @@
       <c r="F73" s="1"/>
       <c r="G73" s="1"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="2">
         <v>2052</v>
       </c>
@@ -7198,7 +7198,7 @@
       <c r="F74" s="1"/>
       <c r="G74" s="1"/>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" s="2">
         <v>2053</v>
       </c>
@@ -7211,7 +7211,7 @@
       <c r="F75" s="1"/>
       <c r="G75" s="1"/>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="2">
         <v>2054</v>
       </c>
@@ -7224,7 +7224,7 @@
       <c r="F76" s="1"/>
       <c r="G76" s="1"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="2">
         <v>2055</v>
       </c>
@@ -7241,7 +7241,7 @@
         <v>82.025000000000006</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" s="2">
         <v>2056</v>
       </c>
@@ -7254,7 +7254,7 @@
       <c r="F78" s="1"/>
       <c r="G78" s="1"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
         <v>2057</v>
       </c>
@@ -7267,7 +7267,7 @@
       <c r="F79" s="1"/>
       <c r="G79" s="1"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" s="2">
         <v>2058</v>
       </c>
@@ -7280,7 +7280,7 @@
       <c r="F80" s="1"/>
       <c r="G80" s="1"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" s="2">
         <v>2059</v>
       </c>
@@ -7293,7 +7293,7 @@
       <c r="F81" s="1"/>
       <c r="G81" s="1"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" s="2">
         <v>2060</v>
       </c>
@@ -7306,7 +7306,7 @@
       <c r="F82" s="1"/>
       <c r="G82" s="1"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" s="2">
         <v>2061</v>
       </c>
@@ -7334,15 +7334,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17725290-58A8-4CE0-98E1-DC575A1B19C6}">
-  <dimension ref="A1:F83"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G83"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="19.42578125" customWidth="1"/>
-    <col min="5" max="5" width="34.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.85546875" customWidth="1"/>
+    <col min="4" max="4" width="19.44140625" customWidth="1"/>
+    <col min="5" max="5" width="34.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7361,8 +7361,11 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1980</v>
       </c>
@@ -7376,7 +7379,7 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>1981</v>
       </c>
@@ -7390,7 +7393,7 @@
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>1982</v>
       </c>
@@ -7404,7 +7407,7 @@
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>1983</v>
       </c>
@@ -7418,7 +7421,7 @@
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>1984</v>
       </c>
@@ -7432,7 +7435,7 @@
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>1985</v>
       </c>
@@ -7446,7 +7449,7 @@
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>1986</v>
       </c>
@@ -7460,7 +7463,7 @@
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>1987</v>
       </c>
@@ -7474,7 +7477,7 @@
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>1988</v>
       </c>
@@ -7488,7 +7491,7 @@
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>1989</v>
       </c>
@@ -7502,7 +7505,7 @@
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>1990</v>
       </c>
@@ -7516,7 +7519,7 @@
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>1991</v>
       </c>
@@ -7530,7 +7533,7 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>1992</v>
       </c>
@@ -7544,7 +7547,7 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>1993</v>
       </c>
@@ -7558,7 +7561,7 @@
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>1994</v>
       </c>
@@ -7572,7 +7575,7 @@
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>1995</v>
       </c>
@@ -7586,7 +7589,7 @@
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>1996</v>
       </c>
@@ -7600,7 +7603,7 @@
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>1997</v>
       </c>
@@ -7614,7 +7617,7 @@
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>1998</v>
       </c>
@@ -7628,7 +7631,7 @@
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>1999</v>
       </c>
@@ -7642,7 +7645,7 @@
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>2000</v>
       </c>
@@ -7656,7 +7659,7 @@
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>2001</v>
       </c>
@@ -7670,7 +7673,7 @@
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>2002</v>
       </c>
@@ -7684,7 +7687,7 @@
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>2003</v>
       </c>
@@ -7698,7 +7701,7 @@
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>2004</v>
       </c>
@@ -7712,7 +7715,7 @@
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>2005</v>
       </c>
@@ -7726,7 +7729,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>2006</v>
       </c>
@@ -7740,7 +7743,7 @@
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>2007</v>
       </c>
@@ -7754,7 +7757,7 @@
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>2008</v>
       </c>
@@ -7768,7 +7771,7 @@
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>2009</v>
       </c>
@@ -7782,7 +7785,7 @@
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>2010</v>
       </c>
@@ -7796,7 +7799,7 @@
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>2011</v>
       </c>
@@ -7810,7 +7813,7 @@
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>2012</v>
       </c>
@@ -7824,7 +7827,7 @@
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>2013</v>
       </c>
@@ -7838,7 +7841,7 @@
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>2014</v>
       </c>
@@ -7852,7 +7855,7 @@
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
         <v>2015</v>
       </c>
@@ -7866,7 +7869,7 @@
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>2016</v>
       </c>
@@ -7880,7 +7883,7 @@
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
         <v>2017</v>
       </c>
@@ -7894,7 +7897,7 @@
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>2018</v>
       </c>
@@ -7908,7 +7911,7 @@
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>2019</v>
       </c>
@@ -7922,7 +7925,7 @@
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>2020</v>
       </c>
@@ -7937,8 +7940,11 @@
       <c r="F42" s="1">
         <v>79</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G42">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <v>2021</v>
       </c>
@@ -7951,7 +7957,7 @@
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
         <v>2022</v>
       </c>
@@ -7964,7 +7970,7 @@
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
         <v>2023</v>
       </c>
@@ -7977,7 +7983,7 @@
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
         <v>2024</v>
       </c>
@@ -7990,7 +7996,7 @@
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <v>2025</v>
       </c>
@@ -8005,8 +8011,11 @@
       <c r="F47" s="1">
         <v>86</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G47">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>2026</v>
       </c>
@@ -8023,7 +8032,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
         <v>2027</v>
       </c>
@@ -8038,7 +8047,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
         <v>2028</v>
       </c>
@@ -8053,7 +8062,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
         <v>2029</v>
       </c>
@@ -8068,7 +8077,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
         <v>2030</v>
       </c>
@@ -8081,8 +8090,11 @@
       <c r="F52" s="1">
         <v>91</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G52">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
         <v>2031</v>
       </c>
@@ -8093,7 +8105,7 @@
       <c r="D53" s="1"/>
       <c r="E53" s="1"/>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
         <v>2032</v>
       </c>
@@ -8104,7 +8116,7 @@
       <c r="D54" s="1"/>
       <c r="E54" s="1"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
         <v>2033</v>
       </c>
@@ -8115,7 +8127,7 @@
       <c r="D55" s="1"/>
       <c r="E55" s="1"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
         <v>2034</v>
       </c>
@@ -8126,7 +8138,7 @@
       <c r="D56" s="1"/>
       <c r="E56" s="1"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
         <v>2035</v>
       </c>
@@ -8139,8 +8151,11 @@
       <c r="F57" s="1">
         <v>92</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G57">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
         <v>2036</v>
       </c>
@@ -8151,7 +8166,7 @@
       <c r="D58" s="1"/>
       <c r="E58" s="1"/>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
         <v>2037</v>
       </c>
@@ -8162,7 +8177,7 @@
       <c r="D59" s="1"/>
       <c r="E59" s="1"/>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
         <v>2038</v>
       </c>
@@ -8173,7 +8188,7 @@
       <c r="D60" s="1"/>
       <c r="E60" s="1"/>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
         <v>2039</v>
       </c>
@@ -8184,7 +8199,7 @@
       <c r="D61" s="1"/>
       <c r="E61" s="1"/>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="2">
         <v>2040</v>
       </c>
@@ -8197,8 +8212,11 @@
       <c r="F62" s="1">
         <v>88</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G62">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
         <v>2041</v>
       </c>
@@ -8209,7 +8227,7 @@
       <c r="D63" s="1"/>
       <c r="E63" s="1"/>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
         <v>2042</v>
       </c>
@@ -8220,7 +8238,7 @@
       <c r="D64" s="1"/>
       <c r="E64" s="1"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
         <v>2043</v>
       </c>
@@ -8231,7 +8249,7 @@
       <c r="D65" s="1"/>
       <c r="E65" s="1"/>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
         <v>2044</v>
       </c>
@@ -8242,7 +8260,7 @@
       <c r="D66" s="1"/>
       <c r="E66" s="1"/>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
         <v>2045</v>
       </c>
@@ -8255,8 +8273,11 @@
       <c r="F67" s="1">
         <v>88</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G67">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" s="2">
         <v>2046</v>
       </c>
@@ -8267,7 +8288,7 @@
       <c r="D68" s="1"/>
       <c r="E68" s="1"/>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
         <v>2047</v>
       </c>
@@ -8278,7 +8299,7 @@
       <c r="D69" s="1"/>
       <c r="E69" s="1"/>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="2">
         <v>2048</v>
       </c>
@@ -8289,7 +8310,7 @@
       <c r="D70" s="1"/>
       <c r="E70" s="1"/>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="2">
         <v>2049</v>
       </c>
@@ -8301,7 +8322,7 @@
       <c r="E71" s="1"/>
       <c r="F71" s="1"/>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="2">
         <v>2050</v>
       </c>
@@ -8314,8 +8335,11 @@
       <c r="F72" s="1">
         <v>89</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G72">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="2">
         <v>2051</v>
       </c>
@@ -8326,7 +8350,7 @@
       <c r="D73" s="1"/>
       <c r="E73" s="1"/>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="2">
         <v>2052</v>
       </c>
@@ -8337,7 +8361,7 @@
       <c r="D74" s="1"/>
       <c r="E74" s="1"/>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" s="2">
         <v>2053</v>
       </c>
@@ -8348,7 +8372,7 @@
       <c r="D75" s="1"/>
       <c r="E75" s="1"/>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="2">
         <v>2054</v>
       </c>
@@ -8359,7 +8383,7 @@
       <c r="D76" s="1"/>
       <c r="E76" s="1"/>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="2">
         <v>2055</v>
       </c>
@@ -8372,8 +8396,11 @@
       <c r="F77" s="1">
         <v>90</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G77">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" s="2">
         <v>2056</v>
       </c>
@@ -8384,7 +8411,7 @@
       <c r="D78" s="1"/>
       <c r="E78" s="1"/>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
         <v>2057</v>
       </c>
@@ -8395,7 +8422,7 @@
       <c r="D79" s="1"/>
       <c r="E79" s="1"/>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" s="2">
         <v>2058</v>
       </c>
@@ -8406,7 +8433,7 @@
       <c r="D80" s="1"/>
       <c r="E80" s="1"/>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" s="2">
         <v>2059</v>
       </c>
@@ -8417,7 +8444,7 @@
       <c r="D81" s="1"/>
       <c r="E81" s="1"/>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" s="2">
         <v>2060</v>
       </c>
@@ -8428,7 +8455,7 @@
       <c r="D82" s="1"/>
       <c r="E82" s="1"/>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" s="2">
         <v>2061</v>
       </c>
@@ -8440,6 +8467,9 @@
       <c r="E83" s="1"/>
       <c r="F83" s="1">
         <v>90</v>
+      </c>
+      <c r="G83">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>